<commit_message>
feat(F-NAR-019): TREE-COL-033 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-COL-033.xlsx
+++ b/stories/arbres/TREE-COL-033.xlsx
@@ -2753,17 +2753,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Nino roule le ballon jusqu'au banc, sable aux genoux. Il s'assoit. Le bois est tiède, comme la chaîne. Le ballon garde la place. Moi, je dis le mot. Il ouvre la bouche trop vite. Papa range le filet. Attends que le filet soit posé, puis toute la phrase. Nino attend. Le ballon ne bouge plus contre le pied. À l'école, près des crochets, une voix a parlé trop près. Ça m'a serré le ventre. La maîtresse m'a donné le galet. Nous t'avons entendu jusqu'au bout. Merci d'avoir attendu. Le galet repose sur une latte, un grain de sable dessus.</t>
+          <t>Nino roule le ballon jusqu'au banc, sable aux genoux. Il s'assoit. Le bois est tiède, comme la chaîne. Le ballon garde la place. Moi, je dis le mot. Il ouvre la bouche trop vite. Papa range le filet. Attends que le filet soit posé, puis toute la phrase. Nino attend. Le ballon ne bouge plus contre le pied. À l'école, près des crochets, une voix a parlé trop près. Ça m'a serré le ventre. La maîtresse m'a donné le galet. Nous t'avons entendu jusqu'au bout. Le galet repose sur une latte, un grain de sable dessus.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino roule le ballon jusqu'au banc, sable aux genoux. Il s'assoit. Le bois est tiède, comme la chaîne. Le ballon garde la place. Moi, je dis le mot. Il ouvre la bouche trop vite. Papa range le filet. Attends que le filet soit posé, puis toute la phrase. Nino attend. Le ballon ne bouge plus contre le pied. À l'école, près des crochets, une voix a parlé trop près. Ça m'a serré le ventre. La maîtresse m'a donné le galet. Nous t'avons entendu jusqu'au bout. Merci d'avoir attendu. Le galet repose sur une &lt;emphasis level="moderate"&gt;latte&lt;/emphasis&gt;, un grain de sable dessus.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino roule le ballon jusqu'au banc, sable aux genoux. Il s'assoit. Le bois est tiède, comme la chaîne. Le ballon garde la place. Moi, je dis le mot. Il ouvre la bouche trop vite. Papa range le filet. Attends que le filet soit posé, puis toute la phrase. Nino attend. Le ballon ne bouge plus contre le pied. À l'école, près des crochets, une voix a parlé trop près. Ça m'a serré le ventre. La maîtresse m'a donné le galet. Nous t'avons entendu jusqu'au bout. Le galet repose sur une &lt;emphasis level="moderate"&gt;latte&lt;/emphasis&gt;, un grain de sable dessus.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Nino roule le ballon jusqu'au banc, sable aux genoux. Il s'assoit. Le bois est tiède, comme la chaîne. Le ballon garde la place. Moi, je dis le mot. Il ouvre la bouche trop vite. Papa range le filet. Attends que le filet soit posé, puis toute la phrase. Nino attend. Le ballon ne bouge plus contre le pied. À l'école, près des crochets, une voix a parlé trop près. Ça m'a serré le ventre. La maîtresse m'a donné le galet. Nous t'avons entendu jusqu'au bout. Merci d'avoir attendu. Le galet repose sur une &lt;emphasis&gt;latte&lt;/emphasis&gt;, un grain de sable dessus. [pause]</t>
+          <t>Nino roule le ballon jusqu'au banc, sable aux genoux. Il s'assoit. Le bois est tiède, comme la chaîne. Le ballon garde la place. Moi, je dis le mot. Il ouvre la bouche trop vite. Papa range le filet. Attends que le filet soit posé, puis toute la phrase. Nino attend. Le ballon ne bouge plus contre le pied. À l'école, près des crochets, une voix a parlé trop près. Ça m'a serré le ventre. La maîtresse m'a donné le galet. Nous t'avons entendu jusqu'au bout. Le galet repose sur une &lt;emphasis&gt;latte&lt;/emphasis&gt;, un grain de sable dessus. [pause]</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -2911,7 +2911,6 @@
 enfant-m|Ça m'a serré le ventre.
 enfant-m|La maîtresse m'a donné le galet.
 papa|Nous t'avons entendu jusqu'au bout.
-papa|Merci d'avoir attendu.
 narrateur|Le galet repose sur une latte, un grain de sable dessus.</t>
         </is>
       </c>
@@ -3131,17 +3130,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Nino essuie le galet contre son short, puis le glisse. La poche sent le sable, et un peu de craie. Il rentre. Le mot aussi. Il parle en marchant. Papa ferme le cartable. On s'arrête. Tes pieds, puis tes mots. Nino s'arrête. Le ballon reste coincé sous son coude. Près des crochets, une voix a parlé trop près. Mon ventre s'est serré. La maîtresse m'a mis le galet là. Merci d'avoir posé tes pieds. Nous avons tout. Un grain de sable reste dans la couture de la poche.</t>
+          <t>Nino essuie le galet contre son short, puis le glisse. La poche sent le sable, et un peu de craie. Il rentre. Le mot aussi. Il parle en marchant. Papa ferme le cartable. On s'arrête. Tes pieds, puis tes mots. Nino s'arrête. Le ballon reste coincé sous son coude. Près des crochets, une voix a parlé trop près. Mon ventre s'est serré. La maîtresse m'a mis le galet là. Tes pieds sont posés. Nous avons toute la phrase. Un grain de sable reste dans la couture de la poche.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino essuie le galet contre son short, puis le glisse. La &lt;emphasis level="moderate"&gt;poche&lt;/emphasis&gt; sent le sable, et un peu de craie. Il rentre. Le mot aussi. Il parle en marchant. Papa ferme le cartable. On s'arrête. Tes pieds, puis tes mots. Nino s'arrête. Le ballon reste coincé sous son coude. Près des crochets, une voix a parlé trop près. Mon ventre s'est serré. La maîtresse m'a mis le galet là. Merci d'avoir posé tes pieds. Nous avons tout. Un grain de sable reste dans la couture de la poche.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino essuie le galet contre son short, puis le glisse. La &lt;emphasis level="moderate"&gt;poche&lt;/emphasis&gt; sent le sable, et un peu de craie. Il rentre. Le mot aussi. Il parle en marchant. Papa ferme le cartable. On s'arrête. Tes pieds, puis tes mots. Nino s'arrête. Le ballon reste coincé sous son coude. Près des crochets, une voix a parlé trop près. Mon ventre s'est serré. La maîtresse m'a mis le galet là. Tes pieds sont posés. Nous avons toute la phrase. Un grain de sable reste dans la couture de la poche.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Nino essuie le galet contre son short, puis le glisse. La &lt;emphasis&gt;poche&lt;/emphasis&gt; sent le sable, et un peu de craie. Il rentre. Le mot aussi. Il parle en marchant. Papa ferme le cartable. On s'arrête. Tes pieds, puis tes mots. Nino s'arrête. Le ballon reste coincé sous son coude. Près des crochets, une voix a parlé trop près. Mon ventre s'est serré. La maîtresse m'a mis le galet là. Merci d'avoir posé tes pieds. Nous avons tout. Un grain de sable reste dans la couture de la poche. [pause]</t>
+          <t>Nino essuie le galet contre son short, puis le glisse. La &lt;emphasis&gt;poche&lt;/emphasis&gt; sent le sable, et un peu de craie. Il rentre. Le mot aussi. Il parle en marchant. Papa ferme le cartable. On s'arrête. Tes pieds, puis tes mots. Nino s'arrête. Le ballon reste coincé sous son coude. Près des crochets, une voix a parlé trop près. Mon ventre s'est serré. La maîtresse m'a mis le galet là. Tes pieds sont posés. Nous avons toute la phrase. Un grain de sable reste dans la couture de la poche. [pause]</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -3288,8 +3287,8 @@
 enfant-m|Près des crochets, une voix a parlé trop près.
 enfant-m|Mon ventre s'est serré.
 enfant-m|La maîtresse m'a mis le galet là.
-maman|Merci d'avoir posé tes pieds.
-maman|Nous avons tout.
+maman|Tes pieds sont posés.
+maman|Nous avons toute la phrase.
 narrateur|Un grain de sable reste dans la couture de la poche.</t>
         </is>
       </c>
@@ -4283,17 +4282,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Nino porte le seau jusqu'au banc, deux mains sur l'anse. Il le pose. Un peu de sable fuit par le fond troué. Le galet est au fond. Le mot est pour le banc. Il s'assoit trop vite. Le seau vacille. On pose l'anse, puis on parle. D'accord ? Nino pose l'anse. Il souffle par le nez. Près des crochets, une voix a parlé trop près. La maîtresse m'a donné le galet. Mon ventre s'est serré. Merci d'avoir posé l'anse. Nous t'écoutions. Le galet reste dans le seau, au pied de la latte.</t>
+          <t>Nino porte le seau jusqu'au banc, deux mains sur l'anse. Il le pose. Un peu de sable fuit par le fond troué. Le galet est au fond. Le mot est pour le banc. Il s'assoit trop vite. Le seau vacille. On pose l'anse, puis on parle. D'accord ? Nino pose l'anse. Il souffle par le nez. Près des crochets, une voix a parlé trop près. La maîtresse m'a donné le galet. Mon ventre s'est serré. L'anse est posée. Nous t'écoutions. Le galet reste dans le seau, au pied de la latte.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino porte le seau jusqu'au banc, deux mains sur l'&lt;emphasis level="moderate"&gt;anse&lt;/emphasis&gt;. Il le pose. Un peu de sable fuit par le fond troué. Le galet est au fond. Le mot est pour le banc. Il s'assoit trop vite. Le seau vacille. On pose l'anse, puis on parle. D'accord ? Nino pose l'anse. Il souffle par le nez. Près des crochets, une voix a parlé trop près. La maîtresse m'a donné le galet. Mon ventre s'est serré. Merci d'avoir posé l'anse. Nous t'écoutions. Le galet reste dans le seau, au pied de la latte.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino porte le seau jusqu'au banc, deux mains sur l'&lt;emphasis level="moderate"&gt;anse&lt;/emphasis&gt;. Il le pose. Un peu de sable fuit par le fond troué. Le galet est au fond. Le mot est pour le banc. Il s'assoit trop vite. Le seau vacille. On pose l'anse, puis on parle. D'accord ? Nino pose l'anse. Il souffle par le nez. Près des crochets, une voix a parlé trop près. La maîtresse m'a donné le galet. Mon ventre s'est serré. L'anse est posée. Nous t'écoutions. Le galet reste dans le seau, au pied de la latte.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Nino porte le seau jusqu'au banc, deux mains sur l'&lt;emphasis&gt;anse&lt;/emphasis&gt;. Il le pose. Un peu de sable fuit par le fond troué. Le galet est au fond. Le mot est pour le banc. Il s'assoit trop vite. Le seau vacille. On pose l'anse, puis on parle. D'accord ? Nino pose l'anse. Il souffle par le nez. Près des crochets, une voix a parlé trop près. La maîtresse m'a donné le galet. Mon ventre s'est serré. Merci d'avoir posé l'anse. Nous t'écoutions. Le galet reste dans le seau, au pied de la latte. [pause]</t>
+          <t>Nino porte le seau jusqu'au banc, deux mains sur l'&lt;emphasis&gt;anse&lt;/emphasis&gt;. Il le pose. Un peu de sable fuit par le fond troué. Le galet est au fond. Le mot est pour le banc. Il s'assoit trop vite. Le seau vacille. On pose l'anse, puis on parle. D'accord ? Nino pose l'anse. Il souffle par le nez. Près des crochets, une voix a parlé trop près. La maîtresse m'a donné le galet. Mon ventre s'est serré. L'anse est posée. Nous t'écoutions. Le galet reste dans le seau, au pied de la latte. [pause]</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -4441,7 +4440,7 @@
 enfant-m|Près des crochets, une voix a parlé trop près.
 enfant-m|La maîtresse m'a donné le galet.
 enfant-m|Mon ventre s'est serré.
-maman|Merci d'avoir posé l'anse.
+maman|L'anse est posée.
 maman|Nous t'écoutions.
 narrateur|Le galet reste dans le seau, au pied de la latte.</t>
         </is>
@@ -5039,17 +5038,17 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Nino tend le seau. Maman avance la paume au-dessus. Le galet tombe, un poids court, dans sa main. Il est à toi le temps du mot. Du sable coule entre ses doigts, fin, blond. On souffle le sable, puis Nino parle. D'accord ? Nino hoche. Il attend le dernier grain. Une voix trop près, aux crochets. Mon ventre s'est serré. La maîtresse a dit de vous le donner, avec la pierre. Merci. Ma paume a le galet. Mes oreilles ont le mot. Un halo de poussière blonde reste sur sa peau.</t>
+          <t>Nino tend le seau. Maman avance la paume au-dessus. Le galet tombe, un poids court, dans sa main. Il est à toi le temps du mot. Du sable coule entre ses doigts, fin, blond. On souffle le sable, puis Nino parle. D'accord ? Nino hoche. Il attend le dernier grain. Une voix trop près, aux crochets. Mon ventre s'est serré. La maîtresse a dit de vous le donner, avec la pierre. Ma paume a le galet. Mes oreilles ont le mot. Un halo de poussière blonde reste sur sa peau.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino tend le seau. Maman avance la paume au-dessus. Le galet tombe, un poids court, dans sa main. Il est à toi le temps du mot. Du sable coule entre ses doigts, fin, blond. On souffle le sable, puis Nino parle. D'accord ? Nino hoche. Il attend le dernier &lt;emphasis level="moderate"&gt;grain&lt;/emphasis&gt;. Une voix trop près, aux crochets. Mon ventre s'est serré. La maîtresse a dit de vous le donner, avec la pierre. Merci. Ma paume a le galet. Mes oreilles ont le mot. Un halo de poussière blonde reste sur sa peau.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino tend le seau. Maman avance la paume au-dessus. Le galet tombe, un poids court, dans sa main. Il est à toi le temps du mot. Du sable coule entre ses doigts, fin, blond. On souffle le sable, puis Nino parle. D'accord ? Nino hoche. Il attend le dernier &lt;emphasis level="moderate"&gt;grain&lt;/emphasis&gt;. Une voix trop près, aux crochets. Mon ventre s'est serré. La maîtresse a dit de vous le donner, avec la pierre. Ma paume a le galet. Mes oreilles ont le mot. Un halo de poussière blonde reste sur sa peau.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Nino tend le seau. Maman avance la paume au-dessus. Le galet tombe, un poids court, dans sa main. Il est à toi le temps du mot. Du sable coule entre ses doigts, fin, blond. On souffle le sable, puis Nino parle. D'accord ? Nino hoche. Il attend le dernier &lt;emphasis&gt;grain&lt;/emphasis&gt;. Une voix trop près, aux crochets. Mon ventre s'est serré. La maîtresse a dit de vous le donner, avec la pierre. Merci. Ma paume a le galet. Mes oreilles ont le mot. Un halo de poussière blonde reste sur sa peau. [pause]</t>
+          <t>Nino tend le seau. Maman avance la paume au-dessus. Le galet tombe, un poids court, dans sa main. Il est à toi le temps du mot. Du sable coule entre ses doigts, fin, blond. On souffle le sable, puis Nino parle. D'accord ? Nino hoche. Il attend le dernier &lt;emphasis&gt;grain&lt;/emphasis&gt;. Une voix trop près, aux crochets. Mon ventre s'est serré. La maîtresse a dit de vous le donner, avec la pierre. Ma paume a le galet. Mes oreilles ont le mot. Un halo de poussière blonde reste sur sa peau. [pause]</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -5195,7 +5194,6 @@
 enfant-m|Une voix trop près, aux crochets.
 enfant-m|Mon ventre s'est serré.
 enfant-m|La maîtresse a dit de vous le donner, avec la pierre.
-maman|Merci.
 maman|Ma paume a le galet.
 maman|Mes oreilles ont le mot.
 narrateur|Un halo de poussière blonde reste sur sa peau.</t>
@@ -6566,17 +6564,17 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Nino met le doudou à cheval sur son bras, comme un témoin. Il dépose le galet dans la paume de papa, sable et tout. Toi tu le tiens. Moi je parle. Papa souffle le grain. Maman range une lanière. La lanière est bouclée. Nous t'écoutons. Nino attendait ce bouclage, lèvres serrées. Une voix trop près, aux crochets. Ça m'a serré. Elle m'a donné le galet. Le doudou a entendu, lui aussi. Ma paume a la pierre. Merci d'avoir attendu la lanière. Le doudou penche vers la main, museau contre le pouce.</t>
+          <t>Nino met le doudou à cheval sur son bras, comme un témoin. Il dépose le galet dans la paume de papa, sable et tout. Toi tu le tiens. Moi je parle. Papa souffle le grain. Maman range une lanière. La lanière est bouclée. Nous t'écoutons. Nino attendait ce bouclage, lèvres serrées. Une voix trop près, aux crochets. Ça m'a serré. Elle m'a donné le galet. Le doudou a entendu, lui aussi. Ma paume a la pierre. La lanière est bouclée. Le doudou penche vers la main, museau contre le pouce.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino met le doudou à cheval sur son bras, comme un témoin. Il dépose le galet dans la paume de papa, sable et tout. Toi tu le tiens. Moi je parle. Papa souffle le grain. Maman range une &lt;emphasis level="moderate"&gt;lanière&lt;/emphasis&gt;. La lanière est bouclée. Nous t'écoutons. Nino attendait ce bouclage, lèvres serrées. Une voix trop près, aux crochets. Ça m'a serré. Elle m'a donné le galet. Le doudou a entendu, lui aussi. Ma paume a la pierre. Merci d'avoir attendu la lanière. Le doudou penche vers la main, museau contre le pouce.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino met le doudou à cheval sur son bras, comme un témoin. Il dépose le galet dans la paume de papa, sable et tout. Toi tu le tiens. Moi je parle. Papa souffle le grain. Maman range une &lt;emphasis level="moderate"&gt;lanière&lt;/emphasis&gt;. La lanière est bouclée. Nous t'écoutons. Nino attendait ce bouclage, lèvres serrées. Une voix trop près, aux crochets. Ça m'a serré. Elle m'a donné le galet. Le doudou a entendu, lui aussi. Ma paume a la pierre. La lanière est bouclée. Le doudou penche vers la main, museau contre le pouce.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Nino met le doudou à cheval sur son bras, comme un témoin. Il dépose le galet dans la paume de papa, sable et tout. Toi tu le tiens. Moi je parle. Papa souffle le grain. Maman range une &lt;emphasis&gt;lanière&lt;/emphasis&gt;. La lanière est bouclée. Nous t'écoutons. Nino attendait ce bouclage, lèvres serrées. Une voix trop près, aux crochets. Ça m'a serré. Elle m'a donné le galet. Le doudou a entendu, lui aussi. Ma paume a la pierre. Merci d'avoir attendu la lanière. Le doudou penche vers la main, museau contre le pouce. [pause]</t>
+          <t>Nino met le doudou à cheval sur son bras, comme un témoin. Il dépose le galet dans la paume de papa, sable et tout. Toi tu le tiens. Moi je parle. Papa souffle le grain. Maman range une &lt;emphasis&gt;lanière&lt;/emphasis&gt;. La lanière est bouclée. Nous t'écoutons. Nino attendait ce bouclage, lèvres serrées. Une voix trop près, aux crochets. Ça m'a serré. Elle m'a donné le galet. Le doudou a entendu, lui aussi. Ma paume a la pierre. La lanière est bouclée. Le doudou penche vers la main, museau contre le pouce. [pause]</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -6724,7 +6722,7 @@
 enfant-m|Elle m'a donné le galet.
 enfant-m|Le doudou a entendu, lui aussi.
 papa|Ma paume a la pierre.
-papa|Merci d'avoir attendu la lanière.
+papa|La lanière est bouclée.
 narrateur|Le doudou penche vers la main, museau contre le pouce.</t>
         </is>
       </c>
@@ -7327,17 +7325,17 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Oui. Il attend que les visages se lèvent. Maman plisse les yeux. Papa lâche la fermeture. Nous te voyons, minuscule, en haut du métal. Le mot n'a pas dévalé. Il est resté avec moi. Merci d'avoir attendu nos visages. Le palier vibre un peu, puis s'arrête. Le galet tient, gris, entre deux genoux.</t>
+          <t>Oui. Il attend que les visages se lèvent. Maman plisse les yeux. Papa lâche la fermeture. Nous te voyons, là-haut, sur le métal. Le mot n'a pas dévalé. Il est resté avec moi. Merci d'avoir attendu nos visages. Le palier vibre un peu, puis s'arrête. Le galet tient, gris, entre deux genoux.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Oui. Il attend que les &lt;emphasis level="moderate"&gt;visages&lt;/emphasis&gt; se lèvent. Maman plisse les yeux. Papa lâche la fermeture. Nous te voyons, minuscule, en haut du métal. Le mot n'a pas dévalé. Il est resté avec moi. Merci d'avoir attendu nos visages. Le palier vibre un peu, puis s'arrête. Le galet tient, gris, entre deux genoux.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Oui. Il attend que les &lt;emphasis level="moderate"&gt;visages&lt;/emphasis&gt; se lèvent. Maman plisse les yeux. Papa lâche la fermeture. Nous te voyons, là-haut, sur le métal. Le mot n'a pas dévalé. Il est resté avec moi. Merci d'avoir attendu nos visages. Le palier vibre un peu, puis s'arrête. Le galet tient, gris, entre deux genoux.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Oui. Il attend que les &lt;emphasis&gt;visages&lt;/emphasis&gt; se lèvent. Maman plisse les yeux. Papa lâche la fermeture. Nous te voyons, minuscule, en haut du métal. Le mot n'a pas dévalé. Il est resté avec moi. Merci d'avoir attendu nos visages. Le palier vibre un peu, puis s'arrête. Le galet tient, gris, entre deux genoux. [pause]</t>
+          <t>Oui. Il attend que les &lt;emphasis&gt;visages&lt;/emphasis&gt; se lèvent. Maman plisse les yeux. Papa lâche la fermeture. Nous te voyons, là-haut, sur le métal. Le mot n'a pas dévalé. Il est resté avec moi. Merci d'avoir attendu nos visages. Le palier vibre un peu, puis s'arrête. Le galet tient, gris, entre deux genoux. [pause]</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
@@ -7475,7 +7473,7 @@
 papa|Il attend que les visages se lèvent.
 narrateur|Maman plisse les yeux.
 narrateur|Papa lâche la fermeture.
-maman|Nous te voyons, minuscule, en haut du métal.
+maman|Nous te voyons, là-haut, sur le métal.
 enfant-m|Le mot n'a pas dévalé.
 enfant-m|Il est resté avec moi.
 papa|Merci d'avoir attendu nos visages.
@@ -8099,17 +8097,17 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Nino descend, le ballon sous le bras, le galet au poing. Ils rejoignent le banc, face à la pente tiède. Le ballon a dévalé tout seul. Le mot, non. Il s'assoit. Le bois craque. Papa souffle. Le craquement d'abord. Après, ta phrase. Nino attend que le bois se taise. En haut, j'ai eu le ventre serré, comme aux crochets. Une voix trop près. La maîtresse m'a donné le galet. Merci d'avoir attendu le banc. Nous avons tout. Le ballon rouge cale un pied de banc, pour ne plus rouler.</t>
+          <t>Nino descend, le ballon sous le bras, le galet au poing. Ils rejoignent le banc, face à la pente tiède. Le ballon a dévalé tout seul. Le mot, non. Il s'assoit. Le bois craque. Papa souffle. Le craquement d'abord. Après, ta phrase. Nino attend que le bois se taise. En haut, j'ai eu le ventre serré, comme aux crochets. Une voix trop près. La maîtresse m'a donné le galet. Le banc s'est tu. Nous avons toute la phrase. Le ballon rouge cale un pied de banc, pour ne plus rouler.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino descend, le ballon sous le bras, le galet au poing. Ils rejoignent le banc, face à la pente tiède. Le ballon a dévalé tout seul. Le mot, non. Il s'assoit. Le bois craque. Papa souffle. Le craquement d'abord. Après, ta phrase. Nino attend que le bois se taise. En haut, j'ai eu le ventre serré, comme aux crochets. Une voix trop près. La maîtresse m'a donné le galet. Merci d'avoir attendu le banc. Nous avons tout. Le ballon rouge cale un pied de banc, pour ne plus rouler.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino descend, le ballon sous le bras, le galet au poing. Ils rejoignent le banc, face à la pente tiède. Le ballon a dévalé tout seul. Le mot, non. Il s'assoit. Le bois craque. Papa souffle. Le craquement d'abord. Après, ta phrase. Nino attend que le bois se taise. En haut, j'ai eu le ventre serré, comme aux crochets. Une voix trop près. La maîtresse m'a donné le galet. Le banc s'est tu. Nous avons toute la phrase. Le ballon rouge cale un pied de banc, pour ne plus rouler.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Nino descend, le ballon sous le bras, le galet au poing. Ils rejoignent le banc, face à la pente tiède. Le ballon a dévalé tout seul. Le mot, non. Il s'assoit. Le bois craque. Papa souffle. Le craquement d'abord. Après, ta phrase. Nino attend que le bois se taise. En haut, j'ai eu le ventre serré, comme aux crochets. Une voix trop près. La maîtresse m'a donné le galet. Merci d'avoir attendu le banc. Nous avons tout. Le ballon rouge cale un pied de banc, pour ne plus rouler. [pause]</t>
+          <t>Nino descend, le ballon sous le bras, le galet au poing. Ils rejoignent le banc, face à la pente tiède. Le ballon a dévalé tout seul. Le mot, non. Il s'assoit. Le bois craque. Papa souffle. Le craquement d'abord. Après, ta phrase. Nino attend que le bois se taise. En haut, j'ai eu le ventre serré, comme aux crochets. Une voix trop près. La maîtresse m'a donné le galet. Le banc s'est tu. Nous avons toute la phrase. Le ballon rouge cale un pied de banc, pour ne plus rouler. [pause]</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -8256,8 +8254,8 @@
 enfant-m|En haut, j'ai eu le ventre serré, comme aux crochets.
 enfant-m|Une voix trop près.
 enfant-m|La maîtresse m'a donné le galet.
-maman|Merci d'avoir attendu le banc.
-maman|Nous avons tout.
+maman|Le banc s'est tu.
+maman|Nous avons toute la phrase.
 narrateur|Le ballon rouge cale un pied de banc, pour ne plus rouler.</t>
         </is>
       </c>
@@ -8857,17 +8855,17 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Maman lève les mains au bas de la pente, paumes ouvertes. Nino, en haut, penche le galet. Il ne le jette pas. Je le pose. Je ne le lance pas. Il descend deux marches. Le galet rejoint la paume. Le ballon attend dans l'herbe, témoin rond. La pierre est arrivée. Maintenant le mot, s'il te plaît ? Nino pose les deux pieds dans l'herbe avant de parler. Une voix trop près, aux crochets. Mon ventre s'est serré. La maîtresse a dit : tu le donnes, ce soir. Tu l'as donné. Merci d'avoir posé tes pieds.</t>
+          <t>Maman lève les mains au bas de la pente, paumes ouvertes. Nino, en haut, penche le galet. Il ne le jette pas. Je le pose. Je ne le lance pas. Il descend deux marches. Le galet rejoint la paume. Le ballon attend dans l'herbe, témoin rond. La pierre est arrivée. Maintenant le mot, s'il te plaît ? Nino pose les deux pieds dans l'herbe avant de parler. Une voix trop près, aux crochets. Mon ventre s'est serré. La maîtresse a dit : tu le donnes, ce soir. Tu l'as donné. Tes pieds sont dans l'herbe.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman lève les mains au bas de la pente, paumes ouvertes. Nino, en haut, penche le galet. Il ne le jette pas. Je le pose. Je ne le lance pas. Il descend deux marches. Le galet rejoint la paume. Le ballon attend dans l'herbe, témoin rond. La pierre est arrivée. Maintenant le mot, s'il te plaît ? Nino pose les deux pieds dans l'herbe avant de parler. Une voix trop près, aux crochets. Mon ventre s'est serré. La maîtresse a dit : tu le donnes, ce soir. Tu l'as donné. Merci d'avoir posé tes pieds.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman lève les mains au bas de la pente, paumes ouvertes. Nino, en haut, penche le galet. Il ne le jette pas. Je le pose. Je ne le lance pas. Il descend deux marches. Le galet rejoint la paume. Le ballon attend dans l'herbe, témoin rond. La pierre est arrivée. Maintenant le mot, s'il te plaît ? Nino pose les deux pieds dans l'herbe avant de parler. Une voix trop près, aux crochets. Mon ventre s'est serré. La maîtresse a dit : tu le donnes, ce soir. Tu l'as donné. Tes pieds sont dans l'herbe.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Maman lève les mains au bas de la pente, paumes ouvertes. Nino, en haut, penche le galet. Il ne le jette pas. Je le pose. Je ne le lance pas. Il descend deux marches. Le galet rejoint la paume. Le ballon attend dans l'herbe, témoin rond. La pierre est arrivée. Maintenant le mot, s'il te plaît ? Nino pose les deux pieds dans l'herbe avant de parler. Une voix trop près, aux crochets. Mon ventre s'est serré. La maîtresse a dit : tu le donnes, ce soir. Tu l'as donné. Merci d'avoir posé tes pieds. [pause]</t>
+          <t>Maman lève les mains au bas de la pente, paumes ouvertes. Nino, en haut, penche le galet. Il ne le jette pas. Je le pose. Je ne le lance pas. Il descend deux marches. Le galet rejoint la paume. Le ballon attend dans l'herbe, témoin rond. La pierre est arrivée. Maintenant le mot, s'il te plaît ? Nino pose les deux pieds dans l'herbe avant de parler. Une voix trop près, aux crochets. Mon ventre s'est serré. La maîtresse a dit : tu le donnes, ce soir. Tu l'as donné. Tes pieds sont dans l'herbe. [pause]</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -9016,7 +9014,7 @@
 enfant-m|Mon ventre s'est serré.
 enfant-m|La maîtresse a dit : tu le donnes, ce soir.
 maman|Tu l'as donné.
-maman|Merci d'avoir posé tes pieds.</t>
+maman|Tes pieds sont dans l'herbe.</t>
         </is>
       </c>
       <c r="AX42" t="inlineStr">
@@ -9629,17 +9627,17 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Papa descend le seau, échelon par échelon, sans le balancer. Ils le portent au banc, le galet coincé au fond. Il n'a pas dévalé. Moi non plus. Nino s'assoit. Il tape l'anse, trop tôt. L'anse se tait, puis tu parles. D'accord ? Il lâche. Le plastique fait un dernier clac. En haut, le ventre, comme aux crochets. Une voix trop près. Elle m'a donné le galet. Le seau l'a gardé. Merci d'avoir laissé le clac. La phrase est entière. Le seau bleu s'adosse au banc, anse vers Nino.</t>
+          <t>Papa descend le seau, échelon par échelon, sans le balancer. Ils le portent au banc, le galet coincé au fond. Il n'a pas dévalé. Moi non plus. Nino s'assoit. Il tape l'anse, trop tôt. L'anse se tait, puis tu parles. D'accord ? Il lâche. Le plastique fait un dernier clac. En haut, le ventre, comme aux crochets. Une voix trop près. Elle m'a donné le galet. Le seau l'a gardé. Le clac est passé. La phrase est entière. Le seau bleu s'adosse au banc, anse vers Nino.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa descend le seau, échelon par échelon, sans le balancer. Ils le portent au banc, le galet coincé au fond. Il n'a pas dévalé. Moi non plus. Nino s'assoit. Il tape l'anse, trop tôt. L'anse se tait, puis tu parles. D'accord ? Il lâche. Le plastique fait un dernier clac. En haut, le ventre, comme aux crochets. Une voix trop près. Elle m'a donné le galet. Le seau l'a gardé. Merci d'avoir laissé le clac. La phrase est entière. Le seau bleu s'adosse au banc, anse vers Nino.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa descend le seau, échelon par échelon, sans le balancer. Ils le portent au banc, le galet coincé au fond. Il n'a pas dévalé. Moi non plus. Nino s'assoit. Il tape l'anse, trop tôt. L'anse se tait, puis tu parles. D'accord ? Il lâche. Le plastique fait un dernier clac. En haut, le ventre, comme aux crochets. Une voix trop près. Elle m'a donné le galet. Le seau l'a gardé. Le clac est passé. La phrase est entière. Le seau bleu s'adosse au banc, anse vers Nino.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Papa descend le seau, échelon par échelon, sans le balancer. Ils le portent au banc, le galet coincé au fond. Il n'a pas dévalé. Moi non plus. Nino s'assoit. Il tape l'anse, trop tôt. L'anse se tait, puis tu parles. D'accord ? Il lâche. Le plastique fait un dernier clac. En haut, le ventre, comme aux crochets. Une voix trop près. Elle m'a donné le galet. Le seau l'a gardé. Merci d'avoir laissé le clac. La phrase est entière. Le seau bleu s'adosse au banc, anse vers Nino. [pause]</t>
+          <t>Papa descend le seau, échelon par échelon, sans le balancer. Ils le portent au banc, le galet coincé au fond. Il n'a pas dévalé. Moi non plus. Nino s'assoit. Il tape l'anse, trop tôt. L'anse se tait, puis tu parles. D'accord ? Il lâche. Le plastique fait un dernier clac. En haut, le ventre, comme aux crochets. Une voix trop près. Elle m'a donné le galet. Le seau l'a gardé. Le clac est passé. La phrase est entière. Le seau bleu s'adosse au banc, anse vers Nino. [pause]</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -9787,7 +9785,7 @@
 enfant-m|Une voix trop près.
 enfant-m|Elle m'a donné le galet.
 enfant-m|Le seau l'a gardé.
-papa|Merci d'avoir laissé le clac.
+papa|Le clac est passé.
 papa|La phrase est entière.
 narrateur|Le seau bleu s'adosse au banc, anse vers Nino.</t>
         </is>
@@ -10387,17 +10385,17 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Papa tient le seau. Maman avance la paume au bord. Nino bascule le fond, un geste court, pas une cascade. Pour ta main. Pas pour l'herbe. Le galet atterrit. La paume se creuse. Un souffle d'air sent le métal du toboggan. Il est arrivé. Tes pieds sont où ? Nino saute du dernier barreau. Deux pieds dans l'herbe. Une voix trop près, aux crochets. Mon ventre s'est serré. Elle a dit de le mettre dans une main de la maison. Ma main est celle-là. Merci d'avoir visé la paume.</t>
+          <t>Papa tient le seau. Maman avance la paume au bord. Nino bascule le fond, un geste court, pas une cascade. Pour ta main. Pas pour l'herbe. Le galet atterrit. La paume se creuse. Un souffle d'air sent le métal du toboggan. Il est arrivé. Tes pieds sont où ? Nino saute du dernier barreau. Deux pieds dans l'herbe. Une voix trop près, aux crochets. Mon ventre s'est serré. Elle a dit de le mettre dans une main de la maison. Ma main est celle-là. Tu as visé la paume.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa tient le seau. Maman avance la paume au bord. Nino bascule le fond, un geste court, pas une cascade. Pour ta main. Pas pour l'herbe. Le galet atterrit. La paume se creuse. Un souffle d'air sent le métal du toboggan. Il est arrivé. Tes pieds sont où ? Nino saute du dernier barreau. Deux pieds dans l'herbe. Une voix trop près, aux crochets. Mon ventre s'est serré. Elle a dit de le mettre dans une main de la maison. Ma main est celle-là. Merci d'avoir visé la paume.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa tient le seau. Maman avance la paume au bord. Nino bascule le fond, un geste court, pas une cascade. Pour ta main. Pas pour l'herbe. Le galet atterrit. La paume se creuse. Un souffle d'air sent le métal du toboggan. Il est arrivé. Tes pieds sont où ? Nino saute du dernier barreau. Deux pieds dans l'herbe. Une voix trop près, aux crochets. Mon ventre s'est serré. Elle a dit de le mettre dans une main de la maison. Ma main est celle-là. Tu as visé la paume.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Papa tient le seau. Maman avance la paume au bord. Nino bascule le fond, un geste court, pas une cascade. Pour ta main. Pas pour l'herbe. Le galet atterrit. La paume se creuse. Un souffle d'air sent le métal du toboggan. Il est arrivé. Tes pieds sont où ? Nino saute du dernier barreau. Deux pieds dans l'herbe. Une voix trop près, aux crochets. Mon ventre s'est serré. Elle a dit de le mettre dans une main de la maison. Ma main est celle-là. Merci d'avoir visé la paume. [pause]</t>
+          <t>Papa tient le seau. Maman avance la paume au bord. Nino bascule le fond, un geste court, pas une cascade. Pour ta main. Pas pour l'herbe. Le galet atterrit. La paume se creuse. Un souffle d'air sent le métal du toboggan. Il est arrivé. Tes pieds sont où ? Nino saute du dernier barreau. Deux pieds dans l'herbe. Une voix trop près, aux crochets. Mon ventre s'est serré. Elle a dit de le mettre dans une main de la maison. Ma main est celle-là. Tu as visé la paume. [pause]</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -10547,7 +10545,7 @@
 enfant-m|Mon ventre s'est serré.
 enfant-m|Elle a dit de le mettre dans une main de la maison.
 maman|Ma main est celle-là.
-maman|Merci d'avoir visé la paume.</t>
+maman|Tu as visé la paume.</t>
         </is>
       </c>
       <c r="AX50" t="inlineStr">
@@ -11537,17 +11535,17 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Dans l'herbe, Nino glisse le galet, puis un bout de doudou. La poche déborde. Une oreille reste dehors. Ils se tiennent. Je peux dire. Un vélo sonne sur la piste. Il parle quand même. On laisse la sonnette. Après, toi. La sonnette file. Nino reprend, main sur l'oreille. Une voix trop près, aux crochets. Ça serrait en haut. Elle m'a donné le galet. Il voyage avec le doudou. Merci d'avoir laissé la sonnette. On a tout. L'échelle jette une ombre en barreaux sur ses chaussures.</t>
+          <t>Dans l'herbe, Nino glisse le galet, puis un bout de doudou. La poche déborde. Une oreille reste dehors. Ils se tiennent. Je peux dire. Un vélo sonne sur la piste. Il parle quand même. On laisse la sonnette. Après, toi. La sonnette file. Nino reprend, main sur l'oreille. Une voix trop près, aux crochets. Ça serrait en haut. Elle m'a donné le galet. Il voyage avec le doudou. La sonnette est partie. On a toute la phrase. L'échelle jette une ombre en barreaux sur ses chaussures.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Dans l'herbe, Nino glisse le galet, puis un bout de doudou. La poche déborde. Une oreille reste dehors. Ils se tiennent. Je peux dire. Un vélo sonne sur la piste. Il parle quand même. On laisse la &lt;emphasis level="moderate"&gt;sonnette&lt;/emphasis&gt;. Après, toi. La sonnette file. Nino reprend, main sur l'oreille. Une voix trop près, aux crochets. Ça serrait en haut. Elle m'a donné le galet. Il voyage avec le doudou. Merci d'avoir laissé la sonnette. On a tout. L'échelle jette une ombre en barreaux sur ses chaussures.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Dans l'herbe, Nino glisse le galet, puis un bout de doudou. La poche déborde. Une oreille reste dehors. Ils se tiennent. Je peux dire. Un vélo sonne sur la piste. Il parle quand même. On laisse la &lt;emphasis level="moderate"&gt;sonnette&lt;/emphasis&gt;. Après, toi. La sonnette file. Nino reprend, main sur l'oreille. Une voix trop près, aux crochets. Ça serrait en haut. Elle m'a donné le galet. Il voyage avec le doudou. La sonnette est partie. On a toute la phrase. L'échelle jette une ombre en barreaux sur ses chaussures.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Dans l'herbe, Nino glisse le galet, puis un bout de doudou. La poche déborde. Une oreille reste dehors. Ils se tiennent. Je peux dire. Un vélo sonne sur la piste. Il parle quand même. On laisse la &lt;emphasis&gt;sonnette&lt;/emphasis&gt;. Après, toi. La sonnette file. Nino reprend, main sur l'oreille. Une voix trop près, aux crochets. Ça serrait en haut. Elle m'a donné le galet. Il voyage avec le doudou. Merci d'avoir laissé la sonnette. On a tout. L'échelle jette une ombre en barreaux sur ses chaussures. [pause]</t>
+          <t>Dans l'herbe, Nino glisse le galet, puis un bout de doudou. La poche déborde. Une oreille reste dehors. Ils se tiennent. Je peux dire. Un vélo sonne sur la piste. Il parle quand même. On laisse la &lt;emphasis&gt;sonnette&lt;/emphasis&gt;. Après, toi. La sonnette file. Nino reprend, main sur l'oreille. Une voix trop près, aux crochets. Ça serrait en haut. Elle m'a donné le galet. Il voyage avec le doudou. La sonnette est partie. On a toute la phrase. L'échelle jette une ombre en barreaux sur ses chaussures. [pause]</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -11696,8 +11694,8 @@
 enfant-m|Ça serrait en haut.
 enfant-m|Elle m'a donné le galet.
 enfant-m|Il voyage avec le doudou.
-maman|Merci d'avoir laissé la sonnette.
-maman|On a tout.
+maman|La sonnette est partie.
+maman|On a toute la phrase.
 narrateur|L'échelle jette une ombre en barreaux sur ses chaussures.</t>
         </is>
       </c>
@@ -11917,17 +11915,17 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Nino garde le doudou. Il pose le galet dans la paume de maman. Le tissu reste sous son nez, une odeur de lessive et de fer. Lui a entendu là-haut. Toi, tu reçois la pierre. Maman ferme les doigts. Papa plie le filet. Le filet est plié. Tes mots peuvent sortir. Nino attendait ce pli. Il lâche le menton du doudou. Aux crochets, une voix trop près. Mon ventre s'est serré. La maîtresse a dit de le poser dans une main, ce soir. C'est fait. Merci d'avoir attendu le filet. Le doudou penche vers la paume, comme pour vérifier.</t>
+          <t>Nino garde le doudou. Il pose le galet dans la paume de maman. Le tissu reste sous son nez, une odeur de lessive et de fer. Lui a entendu là-haut. Toi, tu reçois la pierre. Maman ferme les doigts. Papa plie le filet. Le filet est plié. Tes mots peuvent sortir. Nino attendait ce pli. Il lâche le menton du doudou. Aux crochets, une voix trop près. Mon ventre s'est serré. La maîtresse a dit de le poser dans une main, ce soir. C'est fait. Le filet est plié. Le doudou penche vers la paume, comme pour vérifier.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino garde le doudou. Il pose le galet dans la paume de maman. Le tissu reste sous son nez, une odeur de &lt;emphasis level="moderate"&gt;lessive&lt;/emphasis&gt; et de fer. Lui a entendu là-haut. Toi, tu reçois la pierre. Maman ferme les doigts. Papa plie le filet. Le filet est plié. Tes mots peuvent sortir. Nino attendait ce pli. Il lâche le menton du doudou. Aux crochets, une voix trop près. Mon ventre s'est serré. La maîtresse a dit de le poser dans une main, ce soir. C'est fait. Merci d'avoir attendu le filet. Le doudou penche vers la paume, comme pour vérifier.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino garde le doudou. Il pose le galet dans la paume de maman. Le tissu reste sous son nez, une odeur de &lt;emphasis level="moderate"&gt;lessive&lt;/emphasis&gt; et de fer. Lui a entendu là-haut. Toi, tu reçois la pierre. Maman ferme les doigts. Papa plie le filet. Le filet est plié. Tes mots peuvent sortir. Nino attendait ce pli. Il lâche le menton du doudou. Aux crochets, une voix trop près. Mon ventre s'est serré. La maîtresse a dit de le poser dans une main, ce soir. C'est fait. Le filet est plié. Le doudou penche vers la paume, comme pour vérifier.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Nino garde le doudou. Il pose le galet dans la paume de maman. Le tissu reste sous son nez, une odeur de &lt;emphasis&gt;lessive&lt;/emphasis&gt; et de fer. Lui a entendu là-haut. Toi, tu reçois la pierre. Maman ferme les doigts. Papa plie le filet. Le filet est plié. Tes mots peuvent sortir. Nino attendait ce pli. Il lâche le menton du doudou. Aux crochets, une voix trop près. Mon ventre s'est serré. La maîtresse a dit de le poser dans une main, ce soir. C'est fait. Merci d'avoir attendu le filet. Le doudou penche vers la paume, comme pour vérifier. [pause]</t>
+          <t>Nino garde le doudou. Il pose le galet dans la paume de maman. Le tissu reste sous son nez, une odeur de &lt;emphasis&gt;lessive&lt;/emphasis&gt; et de fer. Lui a entendu là-haut. Toi, tu reçois la pierre. Maman ferme les doigts. Papa plie le filet. Le filet est plié. Tes mots peuvent sortir. Nino attendait ce pli. Il lâche le menton du doudou. Aux crochets, une voix trop près. Mon ventre s'est serré. La maîtresse a dit de le poser dans une main, ce soir. C'est fait. Le filet est plié. Le doudou penche vers la paume, comme pour vérifier. [pause]</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -12076,7 +12074,7 @@
 enfant-m|Mon ventre s'est serré.
 enfant-m|La maîtresse a dit de le poser dans une main, ce soir.
 maman|C'est fait.
-maman|Merci d'avoir attendu le filet.
+maman|Le filet est plié.
 narrateur|Le doudou penche vers la paume, comme pour vérifier.</t>
         </is>
       </c>
@@ -13452,17 +13450,17 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Nino laisse la chaîne. Il pousse le ballon jusqu'au banc. Ils s'assoient face aux balançoires, le poteau un peu loin. Le poum a fini. Le tic aussi. Le mot, maintenant. Un siège vide se balance. Nino parle trop tôt. On attend que le siège s'arrête, puis toute la phrase. Le siège ralentit, s'immobilise, un peu de travers. Aux crochets, une voix trop près. Ça m'a serré le ventre. La maîtresse m'a donné le galet. Je voulais une clochette. Le siège est sage. Merci d'avoir attendu. Le ballon cale le pied du banc. Le galet tient sur une latte.</t>
+          <t>Nino laisse la chaîne. Il pousse le ballon jusqu'au banc. Ils s'assoient face aux balançoires, le poteau un peu loin. Le poum a fini. Le tic aussi. Le mot, maintenant. Un siège vide se balance. Nino parle trop tôt. On attend que le siège s'arrête, puis toute la phrase. Le siège ralentit, s'immobilise, un peu de travers. Aux crochets, une voix trop près. Ça m'a serré le ventre. La maîtresse m'a donné le galet. Je voulais une clochette. Le siège est sage. Ta phrase peut marcher. Le ballon cale le pied du banc. Le galet tient sur une latte.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino laisse la chaîne. Il pousse le ballon jusqu'au banc. Ils s'assoient face aux balançoires, le poteau un peu loin. Le poum a fini. Le tic aussi. Le mot, maintenant. Un siège vide se balance. Nino parle trop tôt. On attend que le siège s'arrête, puis toute la phrase. Le siège ralentit, s'immobilise, un peu de travers. Aux crochets, une voix trop près. Ça m'a serré le ventre. La maîtresse m'a donné le galet. Je voulais une clochette. Le siège est sage. Merci d'avoir attendu. Le ballon cale le pied du banc. Le galet tient sur une latte.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino laisse la chaîne. Il pousse le ballon jusqu'au banc. Ils s'assoient face aux balançoires, le poteau un peu loin. Le poum a fini. Le tic aussi. Le mot, maintenant. Un siège vide se balance. Nino parle trop tôt. On attend que le siège s'arrête, puis toute la phrase. Le siège ralentit, s'immobilise, un peu de travers. Aux crochets, une voix trop près. Ça m'a serré le ventre. La maîtresse m'a donné le galet. Je voulais une clochette. Le siège est sage. Ta phrase peut marcher. Le ballon cale le pied du banc. Le galet tient sur une latte.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Nino laisse la chaîne. Il pousse le ballon jusqu'au banc. Ils s'assoient face aux balançoires, le poteau un peu loin. Le poum a fini. Le tic aussi. Le mot, maintenant. Un siège vide se balance. Nino parle trop tôt. On attend que le siège s'arrête, puis toute la phrase. Le siège ralentit, s'immobilise, un peu de travers. Aux crochets, une voix trop près. Ça m'a serré le ventre. La maîtresse m'a donné le galet. Je voulais une clochette. Le siège est sage. Merci d'avoir attendu. Le ballon cale le pied du banc. Le galet tient sur une latte. [pause]</t>
+          <t>Nino laisse la chaîne. Il pousse le ballon jusqu'au banc. Ils s'assoient face aux balançoires, le poteau un peu loin. Le poum a fini. Le tic aussi. Le mot, maintenant. Un siège vide se balance. Nino parle trop tôt. On attend que le siège s'arrête, puis toute la phrase. Le siège ralentit, s'immobilise, un peu de travers. Aux crochets, une voix trop près. Ça m'a serré le ventre. La maîtresse m'a donné le galet. Je voulais une clochette. Le siège est sage. Ta phrase peut marcher. Le ballon cale le pied du banc. Le galet tient sur une latte. [pause]</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -13611,7 +13609,7 @@
 enfant-m|La maîtresse m'a donné le galet.
 enfant-m|Je voulais une clochette.
 papa|Le siège est sage.
-papa|Merci d'avoir attendu.
+papa|Ta phrase peut marcher.
 narrateur|Le ballon cale le pied du banc.
 narrateur|Le galet tient sur une latte.</t>
         </is>
@@ -14214,17 +14212,17 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Nino prend le galet. Il le pose dans la paume de papa. Le ballon, sous le coude de maman, ne rebondit plus. Pour toi. La chaîne a trop parlé, avant. Papa pèse le gris. Il est plus chaud que le soir. On garde le ballon sage. Nino, tes mots ? Nino pose une main sur la chaîne, sans la bouger. Aux crochets, une voix trop près. Ça serrait. La maîtresse m'a donné ça. Je voulais que ça clique, ici. Ça a cliqué dans ma main. Merci d'avoir posé, pas lancé. Un maillon laisse une marque tiède sur les doigts de Nino.</t>
+          <t>Nino prend le galet. Il le pose dans la paume de papa. Le ballon, sous le coude de maman, ne rebondit plus. Pour toi. La chaîne a trop parlé, avant. Papa pèse le gris. Il est plus chaud que le soir. On garde le ballon sage. Nino, tes mots ? Nino pose une main sur la chaîne, sans la bouger. Aux crochets, une voix trop près. Ça serrait. La maîtresse m'a donné ça. Je voulais que ça clique, ici. Ça a cliqué dans ma main. Tu as posé, pas lancé. Un maillon laisse une marque tiède sur les doigts de Nino.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino prend le galet. Il le pose dans la paume de papa. Le ballon, sous le coude de maman, ne rebondit plus. Pour toi. La chaîne a trop parlé, avant. Papa pèse le gris. Il est plus chaud que le soir. On garde le ballon sage. Nino, tes mots ? Nino pose une main sur la chaîne, sans la bouger. Aux crochets, une voix trop près. Ça serrait. La maîtresse m'a donné ça. Je voulais que ça clique, ici. Ça a cliqué dans ma main. Merci d'avoir posé, pas lancé. Un maillon laisse une &lt;emphasis level="moderate"&gt;marque tiède&lt;/emphasis&gt; sur les doigts de Nino.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino prend le galet. Il le pose dans la paume de papa. Le ballon, sous le coude de maman, ne rebondit plus. Pour toi. La chaîne a trop parlé, avant. Papa pèse le gris. Il est plus chaud que le soir. On garde le ballon sage. Nino, tes mots ? Nino pose une main sur la chaîne, sans la bouger. Aux crochets, une voix trop près. Ça serrait. La maîtresse m'a donné ça. Je voulais que ça clique, ici. Ça a cliqué dans ma main. Tu as posé, pas lancé. Un maillon laisse une &lt;emphasis level="moderate"&gt;marque tiède&lt;/emphasis&gt; sur les doigts de Nino.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Nino prend le galet. Il le pose dans la paume de papa. Le ballon, sous le coude de maman, ne rebondit plus. Pour toi. La chaîne a trop parlé, avant. Papa pèse le gris. Il est plus chaud que le soir. On garde le ballon sage. Nino, tes mots ? Nino pose une main sur la chaîne, sans la bouger. Aux crochets, une voix trop près. Ça serrait. La maîtresse m'a donné ça. Je voulais que ça clique, ici. Ça a cliqué dans ma main. Merci d'avoir posé, pas lancé. Un maillon laisse une &lt;emphasis&gt;marque tiède&lt;/emphasis&gt; sur les doigts de Nino. [pause]</t>
+          <t>Nino prend le galet. Il le pose dans la paume de papa. Le ballon, sous le coude de maman, ne rebondit plus. Pour toi. La chaîne a trop parlé, avant. Papa pèse le gris. Il est plus chaud que le soir. On garde le ballon sage. Nino, tes mots ? Nino pose une main sur la chaîne, sans la bouger. Aux crochets, une voix trop près. Ça serrait. La maîtresse m'a donné ça. Je voulais que ça clique, ici. Ça a cliqué dans ma main. Tu as posé, pas lancé. Un maillon laisse une &lt;emphasis&gt;marque tiède&lt;/emphasis&gt; sur les doigts de Nino. [pause]</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
@@ -14373,7 +14371,7 @@
 enfant-m|La maîtresse m'a donné ça.
 enfant-m|Je voulais que ça clique, ici.
 papa|Ça a cliqué dans ma main.
-papa|Merci d'avoir posé, pas lancé.
+papa|Tu as posé, pas lancé.
 narrateur|Un maillon laisse une marque tiède sur les doigts de Nino.</t>
         </is>
       </c>
@@ -14987,17 +14985,17 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Nino soulève le seau, galet au fond, et gagne le banc. La chaîne, derrière, reste tendue, sans tic. Le seau a attrapé. Le banc va écouter. Il pose trop près du bord. L'anse bascule. Plus au milieu. Après, tes mots. Nino recale. Le bleu s'immobilise entre eux. Une voix trop près, aux crochets. Mon ventre s'est serré. Elle m'a donné le galet. Le seau l'a rattrapé sous le siège. Merci d'avoir recalé. Nous t'écoutions. Une latte du banc a une tache ronde, l'ombre du seau.</t>
+          <t>Nino soulève le seau, galet au fond, et gagne le banc. La chaîne, derrière, reste tendue, sans tic. Le seau a attrapé. Le banc va écouter. Il pose trop près du bord. L'anse bascule. Plus au milieu. Après, tes mots. Nino recale. Le bleu s'immobilise entre eux. Une voix trop près, aux crochets. Mon ventre s'est serré. Elle m'a donné le galet. Le seau l'a rattrapé sous le siège. Le seau est recalé. Nous t'écoutions. Une latte du banc a une tache ronde, l'ombre du seau.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino soulève le seau, galet au fond, et gagne le banc. La chaîne, derrière, reste tendue, sans tic. Le seau a attrapé. Le banc va écouter. Il pose trop près du bord. L'anse bascule. Plus au milieu. Après, tes mots. Nino recale. Le bleu s'immobilise entre eux. Une voix trop près, aux crochets. Mon ventre s'est serré. Elle m'a donné le galet. Le seau l'a rattrapé sous le siège. Merci d'avoir recalé. Nous t'écoutions. Une latte du banc a une &lt;emphasis level="moderate"&gt;tache ronde&lt;/emphasis&gt;, l'ombre du seau.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino soulève le seau, galet au fond, et gagne le banc. La chaîne, derrière, reste tendue, sans tic. Le seau a attrapé. Le banc va écouter. Il pose trop près du bord. L'anse bascule. Plus au milieu. Après, tes mots. Nino recale. Le bleu s'immobilise entre eux. Une voix trop près, aux crochets. Mon ventre s'est serré. Elle m'a donné le galet. Le seau l'a rattrapé sous le siège. Le seau est recalé. Nous t'écoutions. Une latte du banc a une &lt;emphasis level="moderate"&gt;tache ronde&lt;/emphasis&gt;, l'ombre du seau.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Nino soulève le seau, galet au fond, et gagne le banc. La chaîne, derrière, reste tendue, sans tic. Le seau a attrapé. Le banc va écouter. Il pose trop près du bord. L'anse bascule. Plus au milieu. Après, tes mots. Nino recale. Le bleu s'immobilise entre eux. Une voix trop près, aux crochets. Mon ventre s'est serré. Elle m'a donné le galet. Le seau l'a rattrapé sous le siège. Merci d'avoir recalé. Nous t'écoutions. Une latte du banc a une &lt;emphasis&gt;tache ronde&lt;/emphasis&gt;, l'ombre du seau. [pause]</t>
+          <t>Nino soulève le seau, galet au fond, et gagne le banc. La chaîne, derrière, reste tendue, sans tic. Le seau a attrapé. Le banc va écouter. Il pose trop près du bord. L'anse bascule. Plus au milieu. Après, tes mots. Nino recale. Le bleu s'immobilise entre eux. Une voix trop près, aux crochets. Mon ventre s'est serré. Elle m'a donné le galet. Le seau l'a rattrapé sous le siège. Le seau est recalé. Nous t'écoutions. Une latte du banc a une &lt;emphasis&gt;tache ronde&lt;/emphasis&gt;, l'ombre du seau. [pause]</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
@@ -15145,7 +15143,7 @@
 enfant-m|Mon ventre s'est serré.
 enfant-m|Elle m'a donné le galet.
 enfant-m|Le seau l'a rattrapé sous le siège.
-maman|Merci d'avoir recalé.
+maman|Le seau est recalé.
 maman|Nous t'écoutions.
 narrateur|Une latte du banc a une tache ronde, l'ombre du seau.</t>
         </is>
@@ -15749,17 +15747,17 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Nino tend le seau. Papa y plonge la paume, pas les deux. Le galet se pose, un choc sourd, contre la peau. Il est sorti du bleu. Le mot aussi. La chaîne bouge d'un souffle. Nino parle trop tôt. Deux doigts sur le maillon. Puis ta phrase. Nino tient le maillon. Le souffle passe. Une voix trop près, aux crochets. Mon ventre s'est serré. Elle m'a donné ça. Je le mets dans une main, pas par terre. Ma main l'a. Merci d'avoir tenu la chaîne. Le seau vide reste entre ses genoux, léger comme un secret fini.</t>
+          <t>Nino tend le seau. Papa y plonge la paume, pas les deux. Le galet se pose, un choc sourd, contre la peau. Il est sorti du bleu. Le mot aussi. La chaîne bouge d'un souffle. Nino parle trop tôt. Deux doigts sur le maillon. Puis ta phrase. Nino tient le maillon. Le souffle passe. Une voix trop près, aux crochets. Mon ventre s'est serré. Elle m'a donné ça. Je le mets dans une main, pas par terre. Ma main l'a. Tu as tenu la chaîne. Le seau vide reste entre ses genoux, léger comme un secret fini.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino tend le seau. Papa y plonge la paume, pas les deux. Le galet se pose, un &lt;emphasis level="moderate"&gt;choc sourd&lt;/emphasis&gt;, contre la peau. Il est sorti du bleu. Le mot aussi. La chaîne bouge d'un souffle. Nino parle trop tôt. Deux doigts sur le maillon. Puis ta phrase. Nino tient le maillon. Le souffle passe. Une voix trop près, aux crochets. Mon ventre s'est serré. Elle m'a donné ça. Je le mets dans une main, pas par terre. Ma main l'a. Merci d'avoir tenu la chaîne. Le seau vide reste entre ses genoux, léger comme un secret fini.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino tend le seau. Papa y plonge la paume, pas les deux. Le galet se pose, un &lt;emphasis level="moderate"&gt;choc sourd&lt;/emphasis&gt;, contre la peau. Il est sorti du bleu. Le mot aussi. La chaîne bouge d'un souffle. Nino parle trop tôt. Deux doigts sur le maillon. Puis ta phrase. Nino tient le maillon. Le souffle passe. Une voix trop près, aux crochets. Mon ventre s'est serré. Elle m'a donné ça. Je le mets dans une main, pas par terre. Ma main l'a. Tu as tenu la chaîne. Le seau vide reste entre ses genoux, léger comme un secret fini.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Nino tend le seau. Papa y plonge la paume, pas les deux. Le galet se pose, un &lt;emphasis&gt;choc sourd&lt;/emphasis&gt;, contre la peau. Il est sorti du bleu. Le mot aussi. La chaîne bouge d'un souffle. Nino parle trop tôt. Deux doigts sur le maillon. Puis ta phrase. Nino tient le maillon. Le souffle passe. Une voix trop près, aux crochets. Mon ventre s'est serré. Elle m'a donné ça. Je le mets dans une main, pas par terre. Ma main l'a. Merci d'avoir tenu la chaîne. Le seau vide reste entre ses genoux, léger comme un secret fini. [pause]</t>
+          <t>Nino tend le seau. Papa y plonge la paume, pas les deux. Le galet se pose, un &lt;emphasis&gt;choc sourd&lt;/emphasis&gt;, contre la peau. Il est sorti du bleu. Le mot aussi. La chaîne bouge d'un souffle. Nino parle trop tôt. Deux doigts sur le maillon. Puis ta phrase. Nino tient le maillon. Le souffle passe. Une voix trop près, aux crochets. Mon ventre s'est serré. Elle m'a donné ça. Je le mets dans une main, pas par terre. Ma main l'a. Tu as tenu la chaîne. Le seau vide reste entre ses genoux, léger comme un secret fini. [pause]</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -15909,7 +15907,7 @@
 enfant-m|Elle m'a donné ça.
 enfant-m|Je le mets dans une main, pas par terre.
 papa|Ma main l'a.
-papa|Merci d'avoir tenu la chaîne.
+papa|Tu as tenu la chaîne.
 narrateur|Le seau vide reste entre ses genoux, léger comme un secret fini.</t>
         </is>
       </c>
@@ -16519,17 +16517,17 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Nino descend le doudou du siège, galet contre le ventre du tissu. Ils gagnent le banc. La chaîne, seule, fait un arc minuscule. Toi tu n'es plus capitaine. Eux, ils écoutent. Le doudou roule. Nino le rattrape et parle ensemble. L'ami d'abord, assis. Après, toi. Nino cale le doudou entre eux. Il reprend. Aux crochets, une voix trop près. Ça m'a serré. La maîtresse m'a donné le galet. Je le disais au tissu, pas à vous. Maintenant c'est à nous. Merci d'avoir calé l'ami. Une oreille du doudou touche le galet, comme une joue.</t>
+          <t>Nino descend le doudou du siège, galet contre le ventre du tissu. Ils gagnent le banc. La chaîne, seule, fait un arc minuscule. Toi tu n'es plus capitaine. Eux, ils écoutent. Le doudou roule. Nino le rattrape et parle ensemble. L'ami d'abord, assis. Après, toi. Nino cale le doudou entre eux. Il reprend. Aux crochets, une voix trop près. Ça m'a serré. La maîtresse m'a donné le galet. Je le disais au tissu, pas à vous. Maintenant c'est à nous. L'ami est calé. Une oreille du doudou touche le galet, comme une joue.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino descend le doudou du siège, galet contre le ventre du tissu. Ils gagnent le banc. La chaîne, seule, fait un arc minuscule. Toi tu n'es plus &lt;emphasis level="moderate"&gt;capitaine&lt;/emphasis&gt;. Eux, ils écoutent. Le doudou roule. Nino le rattrape et parle ensemble. L'ami d'abord, assis. Après, toi. Nino cale le doudou entre eux. Il reprend. Aux crochets, une voix trop près. Ça m'a serré. La maîtresse m'a donné le galet. Je le disais au tissu, pas à vous. Maintenant c'est à nous. Merci d'avoir calé l'ami. Une oreille du doudou touche le galet, comme une joue.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino descend le doudou du siège, galet contre le ventre du tissu. Ils gagnent le banc. La chaîne, seule, fait un arc minuscule. Toi tu n'es plus &lt;emphasis level="moderate"&gt;capitaine&lt;/emphasis&gt;. Eux, ils écoutent. Le doudou roule. Nino le rattrape et parle ensemble. L'ami d'abord, assis. Après, toi. Nino cale le doudou entre eux. Il reprend. Aux crochets, une voix trop près. Ça m'a serré. La maîtresse m'a donné le galet. Je le disais au tissu, pas à vous. Maintenant c'est à nous. L'ami est calé. Une oreille du doudou touche le galet, comme une joue.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Nino descend le doudou du siège, galet contre le ventre du tissu. Ils gagnent le banc. La chaîne, seule, fait un arc minuscule. Toi tu n'es plus &lt;emphasis&gt;capitaine&lt;/emphasis&gt;. Eux, ils écoutent. Le doudou roule. Nino le rattrape et parle ensemble. L'ami d'abord, assis. Après, toi. Nino cale le doudou entre eux. Il reprend. Aux crochets, une voix trop près. Ça m'a serré. La maîtresse m'a donné le galet. Je le disais au tissu, pas à vous. Maintenant c'est à nous. Merci d'avoir calé l'ami. Une oreille du doudou touche le galet, comme une joue. [pause]</t>
+          <t>Nino descend le doudou du siège, galet contre le ventre du tissu. Ils gagnent le banc. La chaîne, seule, fait un arc minuscule. Toi tu n'es plus &lt;emphasis&gt;capitaine&lt;/emphasis&gt;. Eux, ils écoutent. Le doudou roule. Nino le rattrape et parle ensemble. L'ami d'abord, assis. Après, toi. Nino cale le doudou entre eux. Il reprend. Aux crochets, une voix trop près. Ça m'a serré. La maîtresse m'a donné le galet. Je le disais au tissu, pas à vous. Maintenant c'est à nous. L'ami est calé. Une oreille du doudou touche le galet, comme une joue. [pause]</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr"/>
@@ -16679,7 +16677,7 @@
 enfant-m|La maîtresse m'a donné le galet.
 enfant-m|Je le disais au tissu, pas à vous.
 maman|Maintenant c'est à nous.
-maman|Merci d'avoir calé l'ami.
+maman|L'ami est calé.
 narrateur|Une oreille du doudou touche le galet, comme une joue.</t>
         </is>
       </c>
@@ -17279,17 +17277,17 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Le doudou reste sur le siège, témoin. Nino avance vers maman. Il pose le galet dans sa paume. La chaîne, à côté, ne tic plus. Lui regarde. Toi tu reçois. Moi je dis. Maman hoche. Papa tient le siège pour qu'il ne parte pas. Le siège est tenu. Tes mots peuvent marcher. Nino pose les deux mains derrière le dos, pour ne plus couper. Aux crochets, une voix trop près. Ça m'a serré le ventre. La maîtresse m'a donné le galet. Je le mets dans ta main. Il y est. Merci d'avoir laissé tes mains derrière. Le doudou, sur le siège, penche une oreille vers la paume.</t>
+          <t>Le doudou reste sur le siège, témoin. Nino avance vers maman. Il pose le galet dans sa paume. La chaîne, à côté, ne tic plus. Lui regarde. Toi tu reçois. Moi je dis. Maman hoche. Papa tient le siège pour qu'il ne parte pas. Le siège est tenu. Tes mots peuvent marcher. Nino pose les deux mains derrière le dos, pour ne plus couper. Aux crochets, une voix trop près. Ça m'a serré le ventre. La maîtresse m'a donné le galet. Je le mets dans ta main. Il y est. Tes mains sont restées derrière. Le doudou, sur le siège, penche une oreille vers la paume.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le doudou reste sur le siège, témoin. Nino avance vers maman. Il pose le galet dans sa paume. La chaîne, à côté, ne tic plus. Lui regarde. Toi tu reçois. Moi je dis. Maman hoche. Papa tient le siège pour qu'il ne parte pas. Le siège est tenu. Tes mots peuvent marcher. Nino pose les deux &lt;emphasis level="moderate"&gt;mains derrière&lt;/emphasis&gt; le dos, pour ne plus couper. Aux crochets, une voix trop près. Ça m'a serré le ventre. La maîtresse m'a donné le galet. Je le mets dans ta main. Il y est. Merci d'avoir laissé tes mains derrière. Le doudou, sur le siège, penche une oreille vers la paume.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le doudou reste sur le siège, témoin. Nino avance vers maman. Il pose le galet dans sa paume. La chaîne, à côté, ne tic plus. Lui regarde. Toi tu reçois. Moi je dis. Maman hoche. Papa tient le siège pour qu'il ne parte pas. Le siège est tenu. Tes mots peuvent marcher. Nino pose les deux &lt;emphasis level="moderate"&gt;mains derrière&lt;/emphasis&gt; le dos, pour ne plus couper. Aux crochets, une voix trop près. Ça m'a serré le ventre. La maîtresse m'a donné le galet. Je le mets dans ta main. Il y est. Tes mains sont restées derrière. Le doudou, sur le siège, penche une oreille vers la paume.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Le doudou reste sur le siège, témoin. Nino avance vers maman. Il pose le galet dans sa paume. La chaîne, à côté, ne tic plus. Lui regarde. Toi tu reçois. Moi je dis. Maman hoche. Papa tient le siège pour qu'il ne parte pas. Le siège est tenu. Tes mots peuvent marcher. Nino pose les deux &lt;emphasis&gt;mains derrière&lt;/emphasis&gt; le dos, pour ne plus couper. Aux crochets, une voix trop près. Ça m'a serré le ventre. La maîtresse m'a donné le galet. Je le mets dans ta main. Il y est. Merci d'avoir laissé tes mains derrière. Le doudou, sur le siège, penche une oreille vers la paume. [pause]</t>
+          <t>Le doudou reste sur le siège, témoin. Nino avance vers maman. Il pose le galet dans sa paume. La chaîne, à côté, ne tic plus. Lui regarde. Toi tu reçois. Moi je dis. Maman hoche. Papa tient le siège pour qu'il ne parte pas. Le siège est tenu. Tes mots peuvent marcher. Nino pose les deux &lt;emphasis&gt;mains derrière&lt;/emphasis&gt; le dos, pour ne plus couper. Aux crochets, une voix trop près. Ça m'a serré le ventre. La maîtresse m'a donné le galet. Je le mets dans ta main. Il y est. Tes mains sont restées derrière. Le doudou, sur le siège, penche une oreille vers la paume. [pause]</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -17440,7 +17438,7 @@
 enfant-m|La maîtresse m'a donné le galet.
 enfant-m|Je le mets dans ta main.
 maman|Il y est.
-maman|Merci d'avoir laissé tes mains derrière.
+maman|Tes mains sont restées derrière.
 narrateur|Le doudou, sur le siège, penche une oreille vers la paume.</t>
         </is>
       </c>
@@ -17656,7 +17654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17769,6 +17767,13 @@
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>